<commit_message>
Très Jolie: entrega revisada
</commit_message>
<xml_diff>
--- a/tresjolie-ref/entrega/Calendario-RRSS-Tres-Jolie.xlsx
+++ b/tresjolie-ref/entrega/Calendario-RRSS-Tres-Jolie.xlsx
@@ -13,9 +13,9 @@
     <sheet name="Diciembre" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Octubre'!$A$1:$K$25</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Octubre'!$A$1:$K$26</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Noviembre'!$A$1:$K$21</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Diciembre'!$A$1:$K$25</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Diciembre'!$A$1:$K$24</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -478,7 +478,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Look de la semana (carrusel) + novedad en Google Business</t>
+          <t>Look de la semana (carrusel) + novedad en la ficha de Google</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -613,7 +613,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K25"/>
+  <dimension ref="A1:K26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -767,7 +767,7 @@
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>Recién llegado: Sudadera Badajoz en el probador</t>
+          <t>En el probador: Sudadera Badajoz</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
@@ -777,7 +777,7 @@
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>Recién llegado a la calle Avilés: Sudadera Badajoz. Si te gusta, te lo guardamos 24 h: escríbenos por WhatsApp.</t>
+          <t>Probada en la tienda de la calle Avilés: Sudadera Badajoz. Si te gusta, te la guardamos 24 h: escríbenos por mensaje directo.</t>
         </is>
       </c>
       <c r="I3" s="3" t="inlineStr">
@@ -917,7 +917,7 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>Google Business</t>
+          <t>Ficha de Google</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
@@ -942,7 +942,7 @@
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
-          <t>Esta semana en la tienda de Vallobín: Sudadera Ávila. Tallas S, M, L, XL.</t>
+          <t>Esta semana en la tienda de Vallobín: Sudadera Ávila. Tallas S, M, L.</t>
         </is>
       </c>
       <c r="I6" s="3" t="inlineStr">
@@ -997,7 +997,7 @@
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
-          <t>Primero sola. Luego puesta. Vestido Tarancón, 59,95 €. Quedan tallas S, M, L, XL. #tresjolieoviedo #tresjoliemodalovers #modaoviedo #vallobin #comerciolocal</t>
+          <t>Primero sola. Luego puesta. Vestido Tarancón, 59,95 €. Tallas S, M, L. #tresjolieoviedo #tresjoliemodalovers #modaoviedo #vallobin #comerciolocal</t>
         </is>
       </c>
       <c r="I7" s="3" t="inlineStr">
@@ -1007,7 +1007,7 @@
       </c>
       <c r="J7" s="3" t="inlineStr">
         <is>
-          <t>BAI (montaje con el packshot)</t>
+          <t>BAI (montaje con la foto de la prenda sola)</t>
         </is>
       </c>
       <c r="K7" s="3" t="inlineStr">
@@ -1192,7 +1192,7 @@
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>Google Business</t>
+          <t>Ficha de Google</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
@@ -1207,22 +1207,22 @@
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>Novedad de la semana: Camiseta Murcia</t>
+          <t>Novedad de la semana: Pantalón Cartagena</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>Camiseta Murcia (39,95 €)</t>
+          <t>Pantalón Cartagena (59,95 €)</t>
         </is>
       </c>
       <c r="H11" s="3" t="inlineStr">
         <is>
-          <t>Esta semana en la tienda de Vallobín: Camiseta Murcia. Tallas S, M, L, XL.</t>
+          <t>Esta semana en la tienda de Vallobín: Pantalón Cartagena. Tallas S, M, L. Hoy es festivo: nos vemos mañana.</t>
         </is>
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>Cómo llegar / Llamar</t>
+          <t>Ver la web</t>
         </is>
       </c>
       <c r="J11" s="3" t="inlineStr">
@@ -1272,7 +1272,7 @@
       </c>
       <c r="H12" s="3" t="inlineStr">
         <is>
-          <t>Primero sola. Luego puesta. Sudadera Ávila, 59,95 €. Quedan tallas S, M, L, XL. #tresjolieoviedo #tresjoliemodalovers #modaoviedo #vallobin #comerciolocal</t>
+          <t>Primero sola. Luego puesta. Sudadera Ávila, 59,95 €. Tallas S, M, L. #tresjolieoviedo #tresjoliemodalovers #modaoviedo #vallobin #comerciolocal</t>
         </is>
       </c>
       <c r="I12" s="3" t="inlineStr">
@@ -1282,7 +1282,7 @@
       </c>
       <c r="J12" s="3" t="inlineStr">
         <is>
-          <t>BAI (montaje con el packshot)</t>
+          <t>BAI (montaje con la foto de la prenda sola)</t>
         </is>
       </c>
       <c r="K12" s="3" t="inlineStr">
@@ -1377,7 +1377,7 @@
       </c>
       <c r="G14" s="3" t="inlineStr">
         <is>
-          <t>Shopper Don Algodón Cuero, Bolso Don Algodón I</t>
+          <t>Shopper Don Algodón Cuero, Bolso Don Algodón bandolera</t>
         </is>
       </c>
       <c r="H14" s="3" t="inlineStr">
@@ -1513,21 +1513,21 @@
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>46316</v>
+        <v>46314</v>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>miércoles</t>
+          <t>lunes</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>IG · FB · TikTok</t>
+          <t>Ficha de Google</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>Reel 6–8 s</t>
+          <t>Publicación</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
@@ -1537,27 +1537,27 @@
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>Primero sola, luego puesta: Falda Valencia</t>
+          <t>Novedad de la semana: Sudadera Cáceres Marino</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
         <is>
-          <t>Falda Valencia (54,95 €)</t>
+          <t>Sudadera Cáceres Marino (59,95 €)</t>
         </is>
       </c>
       <c r="H17" s="3" t="inlineStr">
         <is>
-          <t>Primero sola. Luego puesta. Falda Valencia, 54,95 €. Quedan tallas S, M, L, XL. #tresjolieoviedo #tresjoliemodalovers #modaoviedo #vallobin #comerciolocal</t>
+          <t>Esta semana en la tienda de Vallobín: Sudadera Cáceres Marino. Tallas S, M, L.</t>
         </is>
       </c>
       <c r="I17" s="3" t="inlineStr">
         <is>
-          <t>En tienda y en tresjoliemoda.com</t>
+          <t>Cómo llegar / Llamar</t>
         </is>
       </c>
       <c r="J17" s="3" t="inlineStr">
         <is>
-          <t>BAI (montaje con el packshot)</t>
+          <t>BAI</t>
         </is>
       </c>
       <c r="K17" s="3" t="inlineStr">
@@ -1568,51 +1568,51 @@
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>46318</v>
+        <v>46316</v>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>viernes</t>
+          <t>miércoles</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>IG · FB (stories + post)</t>
+          <t>IG · FB · TikTok</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>Foto + stories</t>
+          <t>Reel 6–8 s</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>Oviedo</t>
+          <t>Novedades</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>Hoy es el día: Premios Princesa de Asturias</t>
+          <t>Primero sola, luego puesta: Falda Valencia</t>
         </is>
       </c>
       <c r="G18" s="3" t="inlineStr">
         <is>
-          <t>Vestido Tarancón (59,95 €)</t>
+          <t>Falda Valencia (54,95 €)</t>
         </is>
       </c>
       <c r="H18" s="3" t="inlineStr">
         <is>
-          <t>Hoy Oviedo sale en todas las pantallas. Nosotras, desde Vallobín, con el vestido que mejor le va a un día así.</t>
+          <t>Primero sola. Luego puesta. Falda Valencia, 54,95 €. Tallas S, M, L. #tresjolieoviedo #tresjoliemodalovers #modaoviedo #vallobin #comerciolocal</t>
         </is>
       </c>
       <c r="I18" s="3" t="inlineStr">
         <is>
-          <t>Abrimos hasta las 20:00</t>
+          <t>En tienda y en tresjoliemoda.com</t>
         </is>
       </c>
       <c r="J18" s="3" t="inlineStr">
         <is>
-          <t>Tienda (foto del escaparate)</t>
+          <t>BAI (montaje con la foto de la prenda sola)</t>
         </is>
       </c>
       <c r="K18" s="3" t="inlineStr">
@@ -1623,51 +1623,51 @@
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>46319</v>
+        <v>46318</v>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>sábado</t>
+          <t>viernes</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>IG · FB</t>
+          <t>IG · FB (stories + post)</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>Stories (3–5)</t>
+          <t>Foto + stories</t>
         </is>
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>La tienda</t>
+          <t>Oviedo</t>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>Sábado en la tienda</t>
+          <t>Hoy es el día: Premios Princesa de Asturias</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Vestido Tarancón (59,95 €)</t>
         </is>
       </c>
       <c r="H19" s="3" t="inlineStr">
         <is>
-          <t>Qué hay hoy en tienda, encuesta de "¿esto o esto?" y horario (10:30–14:00).</t>
+          <t>Hoy Oviedo sale en todas las pantallas. Nosotras, desde Vallobín, con el vestido que mejor le va a un día así.</t>
         </is>
       </c>
       <c r="I19" s="3" t="inlineStr">
         <is>
-          <t>Ven a Vallobín</t>
+          <t>Abrimos hasta las 20:00</t>
         </is>
       </c>
       <c r="J19" s="3" t="inlineStr">
         <is>
-          <t>Tienda (móvil, 5 min)</t>
+          <t>Tienda (foto del escaparate)</t>
         </is>
       </c>
       <c r="K19" s="3" t="inlineStr">
@@ -1678,11 +1678,11 @@
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>46321</v>
+        <v>46319</v>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>lunes</t>
+          <t>sábado</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
@@ -1692,37 +1692,37 @@
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>Carrusel</t>
+          <t>Stories (3–5)</t>
         </is>
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>Cómo combinar</t>
+          <t>La tienda</t>
         </is>
       </c>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t>Look de la semana: Sudadera Caceres Marino + Pantalón Vitoria</t>
+          <t>Sábado en la tienda</t>
         </is>
       </c>
       <c r="G20" s="3" t="inlineStr">
         <is>
-          <t>Sudadera Caceres Marino (59,95 €) + Pantalón Vitoria (59,95 €)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H20" s="3" t="inlineStr">
         <is>
-          <t>Una sudadera y una prenda de abajo: tres formas de llevarlo (trabajo, café, cena). ¿Con cuál te quedas?</t>
+          <t>Qué hay hoy en tienda, encuesta de "¿esto o esto?" y horario (10:30–14:00).</t>
         </is>
       </c>
       <c r="I20" s="3" t="inlineStr">
         <is>
-          <t>Desliza → y guarda</t>
+          <t>Ven a Vallobín</t>
         </is>
       </c>
       <c r="J20" s="3" t="inlineStr">
         <is>
-          <t>BAI</t>
+          <t>Tienda (móvil, 5 min)</t>
         </is>
       </c>
       <c r="K20" s="3" t="inlineStr">
@@ -1742,37 +1742,37 @@
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>Google Business</t>
+          <t>IG · FB</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>Publicación</t>
+          <t>Carrusel</t>
         </is>
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>Novedades</t>
+          <t>Cómo combinar</t>
         </is>
       </c>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>Novedad de la semana: Sudadera Caceres Marino</t>
+          <t>Look de la semana: Sudadera Cáceres Marino + Pantalón Vitoria</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
         <is>
-          <t>Sudadera Caceres Marino (59,95 €)</t>
+          <t>Sudadera Cáceres Marino (59,95 €) + Pantalón Vitoria (59,95 €)</t>
         </is>
       </c>
       <c r="H21" s="3" t="inlineStr">
         <is>
-          <t>Esta semana en la tienda de Vallobín: Sudadera Caceres Marino. Tallas S, M, L, XL.</t>
+          <t>Una sudadera y una prenda de abajo: tres formas de llevarlo (trabajo, café, cena). ¿Con cuál te quedas?</t>
         </is>
       </c>
       <c r="I21" s="3" t="inlineStr">
         <is>
-          <t>Cómo llegar / Llamar</t>
+          <t>Desliza → y guarda</t>
         </is>
       </c>
       <c r="J21" s="3" t="inlineStr">
@@ -1788,21 +1788,21 @@
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>46323</v>
+        <v>46321</v>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>miércoles</t>
+          <t>lunes</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>IG · FB · TikTok</t>
+          <t>Ficha de Google</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>Reel 6–8 s</t>
+          <t>Publicación</t>
         </is>
       </c>
       <c r="E22" s="3" t="inlineStr">
@@ -1812,27 +1812,27 @@
       </c>
       <c r="F22" s="3" t="inlineStr">
         <is>
-          <t>Primero sola, luego puesta: Pantalón Cartagena</t>
+          <t>Novedad de la semana: Falda Segovia</t>
         </is>
       </c>
       <c r="G22" s="3" t="inlineStr">
         <is>
-          <t>Pantalón Cartagena (59,95 €)</t>
+          <t>Falda Segovia (54,95 €)</t>
         </is>
       </c>
       <c r="H22" s="3" t="inlineStr">
         <is>
-          <t>Primero sola. Luego puesta. Pantalón Cartagena, 59,95 €. Quedan tallas S, M, L, XL. #tresjolieoviedo #tresjoliemodalovers #modaoviedo #vallobin #comerciolocal</t>
+          <t>Esta semana en la tienda de Vallobín: Falda Segovia. Tallas S, M, L.</t>
         </is>
       </c>
       <c r="I22" s="3" t="inlineStr">
         <is>
-          <t>En tienda y en tresjoliemoda.com</t>
+          <t>Cómo llegar / Llamar</t>
         </is>
       </c>
       <c r="J22" s="3" t="inlineStr">
         <is>
-          <t>BAI (montaje con el packshot)</t>
+          <t>BAI</t>
         </is>
       </c>
       <c r="K22" s="3" t="inlineStr">
@@ -1843,51 +1843,51 @@
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
-        <v>46324</v>
+        <v>46323</v>
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>jueves</t>
+          <t>miércoles</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>IG · FB</t>
+          <t>IG · FB · TikTok</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>Foto / carrusel</t>
+          <t>Reel 6–8 s</t>
         </is>
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>Vosotras</t>
+          <t>Novedades</t>
         </is>
       </c>
       <c r="F23" s="3" t="inlineStr">
         <is>
-          <t>Lo que dicen de nosotras</t>
+          <t>Primero sola, luego puesta: Pantalón Cartagena</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Pantalón Cartagena (59,95 €)</t>
         </is>
       </c>
       <c r="H23" s="3" t="inlineStr">
         <is>
-          <t>5,0 con 47 reseñas en Google. Gracias por cada una. ¿Nos dejas la tuya?</t>
+          <t>Primero sola. Luego puesta. Pantalón Cartagena, 59,95 €. Tallas S, M, L. #tresjolieoviedo #tresjoliemodalovers #modaoviedo #vallobin #comerciolocal</t>
         </is>
       </c>
       <c r="I23" s="3" t="inlineStr">
         <is>
-          <t>Enlace a reseñas</t>
+          <t>En tienda y en tresjoliemoda.com</t>
         </is>
       </c>
       <c r="J23" s="3" t="inlineStr">
         <is>
-          <t>BAI (diseño con una reseña real, con permiso)</t>
+          <t>BAI (montaje con la foto de la prenda sola)</t>
         </is>
       </c>
       <c r="K23" s="3" t="inlineStr">
@@ -1898,51 +1898,51 @@
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
-        <v>46325</v>
+        <v>46324</v>
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>viernes</t>
+          <t>jueves</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>IG · FB · TikTok</t>
+          <t>IG · FB</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>Reel en tienda</t>
+          <t>Foto / carrusel</t>
         </is>
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>La tienda</t>
+          <t>Vosotras</t>
         </is>
       </c>
       <c r="F24" s="3" t="inlineStr">
         <is>
-          <t>Recién llegado: Sudadera Barcelona en el probador</t>
+          <t>Lo que dicen de nosotras</t>
         </is>
       </c>
       <c r="G24" s="3" t="inlineStr">
         <is>
-          <t>Sudadera Barcelona (59,95 €)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H24" s="3" t="inlineStr">
         <is>
-          <t>Recién llegado a la calle Avilés: Sudadera Barcelona. Si te gusta, te lo guardamos 24 h: escríbenos por WhatsApp.</t>
+          <t>5,0 con 47 reseñas en Google. Gracias por cada una. ¿Nos dejas la tuya?</t>
         </is>
       </c>
       <c r="I24" s="3" t="inlineStr">
         <is>
-          <t>Te lo guardamos 24 h</t>
+          <t>Enlace a reseñas</t>
         </is>
       </c>
       <c r="J24" s="3" t="inlineStr">
         <is>
-          <t>Tienda (15 s en el probador)</t>
+          <t>BAI (diseño con una reseña real, con permiso)</t>
         </is>
       </c>
       <c r="K24" s="3" t="inlineStr">
@@ -1953,61 +1953,116 @@
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
+        <v>46325</v>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>viernes</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>IG · FB · TikTok</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>Reel en tienda</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>La tienda</t>
+        </is>
+      </c>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>En el probador: Sudadera Barcelona</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="inlineStr">
+        <is>
+          <t>Sudadera Barcelona (59,95 €)</t>
+        </is>
+      </c>
+      <c r="H25" s="3" t="inlineStr">
+        <is>
+          <t>Probada en la tienda de la calle Avilés: Sudadera Barcelona. Si te gusta, te la guardamos 24 h: escríbenos por mensaje directo.</t>
+        </is>
+      </c>
+      <c r="I25" s="3" t="inlineStr">
+        <is>
+          <t>Te lo guardamos 24 h</t>
+        </is>
+      </c>
+      <c r="J25" s="3" t="inlineStr">
+        <is>
+          <t>Tienda (15 s en el probador)</t>
+        </is>
+      </c>
+      <c r="K25" s="3" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="n">
         <v>46326</v>
       </c>
-      <c r="B25" s="3" t="inlineStr">
+      <c r="B26" s="3" t="inlineStr">
         <is>
           <t>sábado</t>
         </is>
       </c>
-      <c r="C25" s="3" t="inlineStr">
+      <c r="C26" s="3" t="inlineStr">
         <is>
           <t>IG · FB</t>
         </is>
       </c>
-      <c r="D25" s="3" t="inlineStr">
+      <c r="D26" s="3" t="inlineStr">
         <is>
           <t>Stories (3–5)</t>
         </is>
       </c>
-      <c r="E25" s="3" t="inlineStr">
+      <c r="E26" s="3" t="inlineStr">
         <is>
           <t>La tienda</t>
         </is>
       </c>
-      <c r="F25" s="3" t="inlineStr">
+      <c r="F26" s="3" t="inlineStr">
         <is>
           <t>Sábado en la tienda</t>
         </is>
       </c>
-      <c r="G25" s="3" t="inlineStr">
+      <c r="G26" s="3" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H25" s="3" t="inlineStr">
+      <c r="H26" s="3" t="inlineStr">
         <is>
           <t>Qué hay hoy en tienda, encuesta de "¿esto o esto?" y horario (10:30–14:00).</t>
         </is>
       </c>
-      <c r="I25" s="3" t="inlineStr">
+      <c r="I26" s="3" t="inlineStr">
         <is>
           <t>Ven a Vallobín</t>
         </is>
       </c>
-      <c r="J25" s="3" t="inlineStr">
+      <c r="J26" s="3" t="inlineStr">
         <is>
           <t>Tienda (móvil, 5 min)</t>
         </is>
       </c>
-      <c r="K25" s="3" t="inlineStr">
+      <c r="K26" s="3" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K25"/>
+  <autoFilter ref="A1:K26"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2157,7 +2212,7 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Google Business</t>
+          <t>Ficha de Google</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
@@ -2172,22 +2227,22 @@
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>Novedad de la semana: Sudadera Badajoz</t>
+          <t>Novedad de la semana: Sudadera Barcelona</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>Sudadera Badajoz (64,95 €)</t>
+          <t>Sudadera Barcelona (59,95 €)</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>Esta semana en la tienda de Vallobín: Sudadera Badajoz. Tallas S, M, L, XL.</t>
+          <t>Esta semana en la tienda de Vallobín: Sudadera Barcelona. Tallas S, M, L. Hoy es festivo: nos vemos mañana.</t>
         </is>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>Cómo llegar / Llamar</t>
+          <t>Ver la web</t>
         </is>
       </c>
       <c r="J3" s="3" t="inlineStr">
@@ -2237,7 +2292,7 @@
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>Primero sola. Luego puesta. Falda Zamora, 49,95 €. Quedan tallas S, M, L, XL. #tresjolieoviedo #tresjoliemodalovers #modaoviedo #vallobin #comerciolocal</t>
+          <t>Primero sola. Luego puesta. Falda Zamora, 49,95 €. Tallas S, M, L. #tresjolieoviedo #tresjoliemodalovers #modaoviedo #vallobin #comerciolocal</t>
         </is>
       </c>
       <c r="I4" s="3" t="inlineStr">
@@ -2247,7 +2302,7 @@
       </c>
       <c r="J4" s="3" t="inlineStr">
         <is>
-          <t>BAI (montaje con el packshot)</t>
+          <t>BAI (montaje con la foto de la prenda sola)</t>
         </is>
       </c>
       <c r="K4" s="3" t="inlineStr">
@@ -2432,7 +2487,7 @@
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>Google Business</t>
+          <t>Ficha de Google</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
@@ -2447,17 +2502,17 @@
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>Novedad de la semana: Sudadera Barcelona</t>
+          <t>Novedad de la semana: Falda Valencia</t>
         </is>
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
-          <t>Sudadera Barcelona (59,95 €)</t>
+          <t>Falda Valencia (54,95 €)</t>
         </is>
       </c>
       <c r="H8" s="3" t="inlineStr">
         <is>
-          <t>Esta semana en la tienda de Vallobín: Sudadera Barcelona. Tallas S, M, L, XL.</t>
+          <t>Esta semana en la tienda de Vallobín: Falda Valencia. Tallas S, M, L.</t>
         </is>
       </c>
       <c r="I8" s="3" t="inlineStr">
@@ -2512,7 +2567,7 @@
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
-          <t>Primero sola. Luego puesta. Sudadera Badajoz, 64,95 €. Quedan tallas S, M, L, XL. #tresjolieoviedo #tresjoliemodalovers #modaoviedo #vallobin #comerciolocal</t>
+          <t>Primero sola. Luego puesta. Sudadera Badajoz, 64,95 €. Tallas S, M, L. #tresjolieoviedo #tresjoliemodalovers #modaoviedo #vallobin #comerciolocal</t>
         </is>
       </c>
       <c r="I9" s="3" t="inlineStr">
@@ -2522,7 +2577,7 @@
       </c>
       <c r="J9" s="3" t="inlineStr">
         <is>
-          <t>BAI (montaje con el packshot)</t>
+          <t>BAI (montaje con la foto de la prenda sola)</t>
         </is>
       </c>
       <c r="K9" s="3" t="inlineStr">
@@ -2612,17 +2667,17 @@
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>Recién llegado: Sudadera Caceres Marino en el probador</t>
+          <t>En el probador: Sudadera Cáceres Marino</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>Sudadera Caceres Marino (59,95 €)</t>
+          <t>Sudadera Cáceres Marino (59,95 €)</t>
         </is>
       </c>
       <c r="H11" s="3" t="inlineStr">
         <is>
-          <t>Recién llegado a la calle Avilés: Sudadera Caceres Marino. Si te gusta, te lo guardamos 24 h: escríbenos por WhatsApp.</t>
+          <t>Probada en la tienda de la calle Avilés: Sudadera Cáceres Marino. Si te gusta, te la guardamos 24 h: escríbenos por mensaje directo.</t>
         </is>
       </c>
       <c r="I11" s="3" t="inlineStr">
@@ -2732,12 +2787,12 @@
       </c>
       <c r="H13" s="3" t="inlineStr">
         <is>
-          <t>El Black Friday llega el 27, pero quien esté en nuestra lista lo sabrá antes. Escríbenos "LISTA" por WhatsApp o apúntate en la web.</t>
+          <t>El Black Friday llega el 27, pero quien esté en nuestra lista lo sabrá antes. Escríbenos "LISTA" por mensaje directo o apúntate en la web.</t>
         </is>
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>WhatsApp / boletín</t>
+          <t>Mensaje directo / boletín</t>
         </is>
       </c>
       <c r="J13" s="3" t="inlineStr">
@@ -2787,7 +2842,7 @@
       </c>
       <c r="H14" s="3" t="inlineStr">
         <is>
-          <t>Primero sola. Luego puesta. Camiseta Murcia, 39,95 €. Quedan tallas S, M, L, XL. #tresjolieoviedo #tresjoliemodalovers #modaoviedo #vallobin #comerciolocal</t>
+          <t>Primero sola. Luego puesta. Camiseta Murcia, 39,95 €. Tallas S, M, L. #tresjolieoviedo #tresjoliemodalovers #modaoviedo #vallobin #comerciolocal</t>
         </is>
       </c>
       <c r="I14" s="3" t="inlineStr">
@@ -2797,7 +2852,7 @@
       </c>
       <c r="J14" s="3" t="inlineStr">
         <is>
-          <t>BAI (montaje con el packshot)</t>
+          <t>BAI (montaje con la foto de la prenda sola)</t>
         </is>
       </c>
       <c r="K14" s="3" t="inlineStr">
@@ -2837,7 +2892,7 @@
       </c>
       <c r="G15" s="3" t="inlineStr">
         <is>
-          <t>Shopper Don Algodón Cuero, Bolso Don Algodón I</t>
+          <t>Shopper Don Algodón Cuero, Bolso Don Algodón bandolera</t>
         </is>
       </c>
       <c r="H15" s="3" t="inlineStr">
@@ -2997,7 +3052,7 @@
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>Lo más pedido del año, sola y puesta</t>
+          <t>Dos favoritas del otoño, solas y puestas</t>
         </is>
       </c>
       <c r="G18" s="3" t="inlineStr">
@@ -3007,7 +3062,7 @@
       </c>
       <c r="H18" s="3" t="inlineStr">
         <is>
-          <t>Las dos prendas que más nos habéis preguntado este otoño. Primero solas, luego puestas.</t>
+          <t>Dos de nuestras favoritas de este otoño, ahora en Black Week. Primero solas, luego puestas.</t>
         </is>
       </c>
       <c r="I18" s="3" t="inlineStr">
@@ -3017,7 +3072,7 @@
       </c>
       <c r="J18" s="3" t="inlineStr">
         <is>
-          <t>BAI (packshots) + tienda</t>
+          <t>BAI (fotos de la prenda sola) + tienda</t>
         </is>
       </c>
       <c r="K18" s="3" t="inlineStr">
@@ -3203,7 +3258,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K25"/>
+  <dimension ref="A1:K24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -3367,7 +3422,7 @@
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>Primero sola. Luego puesta. Falda Lely, 54,95 €. Quedan tallas S, M, L, XL. #tresjolieoviedo #tresjoliemodalovers #modaoviedo #vallobin #comerciolocal</t>
+          <t>Primero sola. Luego puesta. Falda Lely, 54,95 €. Tallas S, M, L. #tresjolieoviedo #tresjoliemodalovers #modaoviedo #vallobin #comerciolocal</t>
         </is>
       </c>
       <c r="I3" s="3" t="inlineStr">
@@ -3377,7 +3432,7 @@
       </c>
       <c r="J3" s="3" t="inlineStr">
         <is>
-          <t>BAI (montaje con el packshot)</t>
+          <t>BAI (montaje con la foto de la prenda sola)</t>
         </is>
       </c>
       <c r="K3" s="3" t="inlineStr">
@@ -3417,7 +3472,7 @@
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>Shopper Don Algodón Cuero (61,99 €), Bolso Don Algodón I (49,99 €), Bolso Don Algodón II (69,99 €)</t>
+          <t>Shopper Don Algodón Cuero (61,99 €), Bolso Don Algodón bandolera (49,99 €), Bolso Don Algodón de hombro (69,99 €)</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
@@ -3537,7 +3592,7 @@
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>Compra online o ven el martes</t>
+          <t>Compra online o ven el miércoles 9 (lunes 7 y martes 8, festivos)</t>
         </is>
       </c>
       <c r="J6" s="3" t="inlineStr">
@@ -3587,7 +3642,7 @@
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
-          <t>Primero sola. Luego puesta. Pantalón Vitoria, 59,95 €. Quedan tallas S, M, L, XL. #tresjolieoviedo #tresjoliemodalovers #modaoviedo #vallobin #comerciolocal</t>
+          <t>Primero sola. Luego puesta. Pantalón Vitoria, 59,95 €. Tallas S, M, L. #tresjolieoviedo #tresjoliemodalovers #modaoviedo #vallobin #comerciolocal</t>
         </is>
       </c>
       <c r="I7" s="3" t="inlineStr">
@@ -3597,7 +3652,7 @@
       </c>
       <c r="J7" s="3" t="inlineStr">
         <is>
-          <t>BAI (montaje con el packshot)</t>
+          <t>BAI (montaje con la foto de la prenda sola)</t>
         </is>
       </c>
       <c r="K7" s="3" t="inlineStr">
@@ -3687,7 +3742,7 @@
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>Recién llegado: Sudadera Ávila en el probador</t>
+          <t>En el probador: Sudadera Ávila</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
@@ -3697,7 +3752,7 @@
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
-          <t>Recién llegado a la calle Avilés: Sudadera Ávila. Si te gusta, te lo guardamos 24 h: escríbenos por WhatsApp.</t>
+          <t>Probada en la tienda de la calle Avilés: Sudadera Ávila. Si te gusta, te la guardamos 24 h: escríbenos por mensaje directo.</t>
         </is>
       </c>
       <c r="I9" s="3" t="inlineStr">
@@ -3837,7 +3892,7 @@
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>Google Business</t>
+          <t>Ficha de Google</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
@@ -3852,17 +3907,17 @@
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>Novedad de la semana: Camiseta Murcia</t>
+          <t>Novedad de la semana: Sudadera Ávila</t>
         </is>
       </c>
       <c r="G12" s="3" t="inlineStr">
         <is>
-          <t>Camiseta Murcia (39,95 €)</t>
+          <t>Sudadera Ávila (59,95 €)</t>
         </is>
       </c>
       <c r="H12" s="3" t="inlineStr">
         <is>
-          <t>Esta semana en la tienda de Vallobín: Camiseta Murcia. Tallas S, M, L, XL.</t>
+          <t>Esta semana en la tienda de Vallobín: Sudadera Ávila. Tallas S, M, L.</t>
         </is>
       </c>
       <c r="I12" s="3" t="inlineStr">
@@ -4087,7 +4142,7 @@
       </c>
       <c r="I16" s="3" t="inlineStr">
         <is>
-          <t>Pídela en tienda o por WhatsApp</t>
+          <t>Pídela en tienda o por mensaje directo</t>
         </is>
       </c>
       <c r="J16" s="3" t="inlineStr">
@@ -4103,21 +4158,21 @@
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>46379</v>
+        <v>46377</v>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>miércoles</t>
+          <t>lunes</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>IG · FB · TikTok</t>
+          <t>Ficha de Google</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>Reel 6–8 s</t>
+          <t>Publicación</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
@@ -4127,27 +4182,27 @@
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>Primero sola, luego puesta: Sudadera Barcelona</t>
+          <t>Novedad de la semana: Falda Valencia</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
         <is>
-          <t>Sudadera Barcelona (59,95 €)</t>
+          <t>Falda Valencia (54,95 €)</t>
         </is>
       </c>
       <c r="H17" s="3" t="inlineStr">
         <is>
-          <t>Primero sola. Luego puesta. Sudadera Barcelona, 59,95 €. Quedan tallas S, M, L, XL. #tresjolieoviedo #tresjoliemodalovers #modaoviedo #vallobin #comerciolocal</t>
+          <t>Esta semana en la tienda de Vallobín: Falda Valencia. Tallas S, M, L.</t>
         </is>
       </c>
       <c r="I17" s="3" t="inlineStr">
         <is>
-          <t>En tienda y en tresjoliemoda.com</t>
+          <t>Cómo llegar / Llamar</t>
         </is>
       </c>
       <c r="J17" s="3" t="inlineStr">
         <is>
-          <t>BAI (montaje con el packshot)</t>
+          <t>BAI</t>
         </is>
       </c>
       <c r="K17" s="3" t="inlineStr">
@@ -4158,51 +4213,51 @@
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>46380</v>
+        <v>46379</v>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>jueves</t>
+          <t>miércoles</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>IG · FB</t>
+          <t>IG · FB · TikTok</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>Foto / carrusel</t>
+          <t>Reel 6–8 s</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>Vosotras</t>
+          <t>Novedades</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>Lo que dicen de nosotras</t>
+          <t>Primero sola, luego puesta: Sudadera Barcelona</t>
         </is>
       </c>
       <c r="G18" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Sudadera Barcelona (59,95 €)</t>
         </is>
       </c>
       <c r="H18" s="3" t="inlineStr">
         <is>
-          <t>5,0 con 47 reseñas en Google. Gracias por cada una. ¿Nos dejas la tuya?</t>
+          <t>Primero sola. Luego puesta. Sudadera Barcelona, 59,95 €. Tallas S, M, L. #tresjolieoviedo #tresjoliemodalovers #modaoviedo #vallobin #comerciolocal</t>
         </is>
       </c>
       <c r="I18" s="3" t="inlineStr">
         <is>
-          <t>Enlace a reseñas</t>
+          <t>En tienda y en tresjoliemoda.com</t>
         </is>
       </c>
       <c r="J18" s="3" t="inlineStr">
         <is>
-          <t>BAI (diseño con una reseña real, con permiso)</t>
+          <t>BAI (montaje con la foto de la prenda sola)</t>
         </is>
       </c>
       <c r="K18" s="3" t="inlineStr">
@@ -4213,51 +4268,51 @@
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>46381</v>
+        <v>46380</v>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>viernes</t>
+          <t>jueves</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>IG · FB · TikTok</t>
+          <t>IG · FB</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>Reel en tienda</t>
+          <t>Foto / carrusel</t>
         </is>
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>La tienda</t>
+          <t>Vosotras</t>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>Recién llegado: Falda Valencia en el probador</t>
+          <t>Lo que dicen de nosotras</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
         <is>
-          <t>Falda Valencia (54,95 €)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H19" s="3" t="inlineStr">
         <is>
-          <t>Recién llegado a la calle Avilés: Falda Valencia. Si te gusta, te lo guardamos 24 h: escríbenos por WhatsApp.</t>
+          <t>5,0 con 47 reseñas en Google. Gracias por cada una. ¿Nos dejas la tuya?</t>
         </is>
       </c>
       <c r="I19" s="3" t="inlineStr">
         <is>
-          <t>Te lo guardamos 24 h</t>
+          <t>Enlace a reseñas</t>
         </is>
       </c>
       <c r="J19" s="3" t="inlineStr">
         <is>
-          <t>Tienda (15 s en el probador)</t>
+          <t>BAI (diseño con una reseña real, con permiso)</t>
         </is>
       </c>
       <c r="K19" s="3" t="inlineStr">
@@ -4307,7 +4362,7 @@
       </c>
       <c r="I20" s="3" t="inlineStr">
         <is>
-          <t>Abrimos el lunes 28</t>
+          <t>En tienda y en tresjoliemoda.com</t>
         </is>
       </c>
       <c r="J20" s="3" t="inlineStr">
@@ -4387,7 +4442,7 @@
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>Google Business</t>
+          <t>Ficha de Google</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
@@ -4402,17 +4457,17 @@
       </c>
       <c r="F22" s="3" t="inlineStr">
         <is>
-          <t>Novedad de la semana: Sudadera Ávila</t>
+          <t>Novedad de la semana: Camiseta Murcia</t>
         </is>
       </c>
       <c r="G22" s="3" t="inlineStr">
         <is>
-          <t>Sudadera Ávila (59,95 €)</t>
+          <t>Camiseta Murcia (39,95 €)</t>
         </is>
       </c>
       <c r="H22" s="3" t="inlineStr">
         <is>
-          <t>Esta semana en la tienda de Vallobín: Sudadera Ávila. Tallas S, M, L, XL.</t>
+          <t>Esta semana en la tienda de Vallobín: Camiseta Murcia. Tallas S, M, L.</t>
         </is>
       </c>
       <c r="I22" s="3" t="inlineStr">
@@ -4488,51 +4543,51 @@
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
-        <v>46386</v>
+        <v>46387</v>
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>miércoles</t>
+          <t>jueves</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>IG · FB · TikTok</t>
+          <t>IG · FB</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>Reel 6–8 s</t>
+          <t>Foto</t>
         </is>
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>Novedades</t>
+          <t>Vosotras</t>
         </is>
       </c>
       <c r="F24" s="3" t="inlineStr">
         <is>
-          <t>Primero sola, luego puesta: Falda Segovia</t>
+          <t>Gracias por 2026</t>
         </is>
       </c>
       <c r="G24" s="3" t="inlineStr">
         <is>
-          <t>Falda Segovia (54,95 €)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H24" s="3" t="inlineStr">
         <is>
-          <t>Primero sola. Luego puesta. Falda Segovia, 54,95 €. Quedan tallas S, M, L, XL. #tresjolieoviedo #tresjoliemodalovers #modaoviedo #vallobin #comerciolocal</t>
+          <t>Gracias a cada clienta que ha pasado por la calle Avilés este año. El 7 de enero, rebajas.</t>
         </is>
       </c>
       <c r="I24" s="3" t="inlineStr">
         <is>
-          <t>En tienda y en tresjoliemoda.com</t>
+          <t>Nos vemos en enero</t>
         </is>
       </c>
       <c r="J24" s="3" t="inlineStr">
         <is>
-          <t>BAI (montaje con el packshot)</t>
+          <t>Tienda (foto de equipo)</t>
         </is>
       </c>
       <c r="K24" s="3" t="inlineStr">
@@ -4541,63 +4596,8 @@
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="2" t="n">
-        <v>46387</v>
-      </c>
-      <c r="B25" s="3" t="inlineStr">
-        <is>
-          <t>jueves</t>
-        </is>
-      </c>
-      <c r="C25" s="3" t="inlineStr">
-        <is>
-          <t>IG · FB</t>
-        </is>
-      </c>
-      <c r="D25" s="3" t="inlineStr">
-        <is>
-          <t>Foto</t>
-        </is>
-      </c>
-      <c r="E25" s="3" t="inlineStr">
-        <is>
-          <t>Vosotras</t>
-        </is>
-      </c>
-      <c r="F25" s="3" t="inlineStr">
-        <is>
-          <t>Gracias por 2026</t>
-        </is>
-      </c>
-      <c r="G25" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H25" s="3" t="inlineStr">
-        <is>
-          <t>Gracias a cada clienta que ha pasado por la calle Avilés este año. El 7 de enero, rebajas.</t>
-        </is>
-      </c>
-      <c r="I25" s="3" t="inlineStr">
-        <is>
-          <t>Nos vemos en enero</t>
-        </is>
-      </c>
-      <c r="J25" s="3" t="inlineStr">
-        <is>
-          <t>Tienda (foto de equipo)</t>
-        </is>
-      </c>
-      <c r="K25" s="3" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:K25"/>
+  <autoFilter ref="A1:K24"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>